<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.001-08 Sarah répète et laisse observer
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.001-08.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.001-08.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le bateau dans la bassine</t>
+          <t>Sarah répète et laisse observer</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin, cabanon, fin d'après-midi</t>
+          <t>classe, tapis vert roulé, boîte en fer, anneaux, cour et marché loin, pain près de la fenêtre</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, Victorino, papa, maman</t>
+          <t>Sarah, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut que le bateau de bois traverse la bassine. Victorino reste près de la porte du cabanon. Elle répète : on pousse, puis on attend. Il observe d'abord. Sur la serviette, même jeu. Le bateau touche l'autre bord.</t>
+          <t>Ça sent le pain chaud près de la fenêtre. Un éclat de cour glisse sur le sol. Sarah veut le tapis et tous les anneaux maintenant. Elle verse trop vite : les anneaux glissent. Sourire parti. Elle refuse de foncer, dit un anneau puis un autre. Merci vécu. Le tapis trop vite cache l'éclat. Un éclat de cour reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La mousse du robinet sent le bois mouillé. Une goutte tombe dans la bassine. Elle fait un petit rond. Le soleil est bas, tout orange. Le cabanon a une porte peinte en vert. La peinture s'écaille un peu. Un bateau de bois flotte, tout léger. Sa voile est un carré de tissu. Tu as vu le rond, Sarah ? Oui, maman. Il grandit, puis il part. L'eau est tiède, ce soir. Je veux qu'il traverse. Jusqu'à l'autre bord. Avec la voile ? Oui. En ce moment, Sarah touche le bateau. Le bois est lisse et humide. Victorino reste près de la porte. Il tient le bord du cabanon. Il a besoin de calme. Victorino. Tu pousses avec moi ? Victorino ne vient pas encore. On peut répéter, tout doux. On peut observer d'abord. D'accord. Une feuille tombe dans l'eau. Elle devient une petite île. Tu as vu la feuille, Sarah ? Oui. Le bateau peut tourner autour. Oui. Sans presser. Sarah pose un doigt sur l'eau. L'eau est tiède, comme papa a dit. Victorino regarde depuis la porte. Ses pieds restent sur la pierre.</t>
+          <t>Ça sent le pain chaud, près de la fenêtre. Le marché parle, tout loin. J'entends le pain, papa. Tu l'entends, Sarah ? Un éclat de cour glisse sur le sol. Il brille, papa. Tu le vois, près de la fenêtre ? Sarah touche l'éclat de cour. Le sol est lisse, un peu froid. Il est froid. Maman noue le lacet de Sarah. Ton lacet va là, près de la chaussure. Il tient, maman. La chaussure sent un peu la cour. Elle est froide, maman. Une boîte en fer attend sous la fenêtre. Des anneaux s'y cognent. Ça fait clic. Tu tiens ma manche, Sarah ? Oui, papa. Le tapis vert est roulé dans le coin. Un coin de laine dépasse, un peu rêche. Il est vert, maman. Il sent la laine. Ça pique un peu. Papa pose la bouteille sur l'étagère. L'eau va là. Elle est haute. La bouteille claque contre l'étagère. L'air de la cour entre un peu. J'ai les joues froides. On avance. Tu restes près de nous ? Oui, maman. Je veux le tapis, maintenant ! Tous les anneaux, d'un coup ! Tu ouvres la boîte ? Oui, papa. En ce moment, Sarah ouvre la boîte. Les anneaux sentent le fer. Ils sont froids. Sarah verse trop vite, trop fort. Les anneaux glissent sur le sol. Oh. L'éclat n'est plus là. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je les prends ! Les anneaux sont partout. Tu les vois, Sarah ? Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La mousse du robinet sent le bois mouillé. Une goutte tombe dans la bassine. Elle fait un petit rond. Le soleil est bas, tout orange. Le cabanon a une porte peinte en vert. La peinture s'écaille un peu. Un bateau de bois flotte, tout léger. Sa voile est un carré de tissu. Tu as vu le rond, Sarah ? Oui, maman. Il grandit, puis il part. L'eau est tiède, ce soir. Je veux qu'il traverse. Jusqu'à l'autre bord. Avec la voile ? Oui. En ce moment, Sarah touche le bateau. Le bois est lisse et humide. Victorino reste près de la porte. Il tient le bord du cabanon. Il a besoin de calme. Victorino. Tu pousses avec moi ? Victorino ne vient pas encore. On peut répéter, tout doux. On peut observer d'abord. D'accord. Une feuille tombe dans l'eau. Elle devient une petite île. Tu as vu la feuille, Sarah ? Oui. Le bateau peut tourner autour. Oui. Sans presser. Sarah pose un doigt sur l'eau. L'eau est tiède, comme papa a dit. Victorino regarde depuis la porte. Ses pieds restent sur la pierre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ça sent le pain chaud, près de la fenêtre. Le marché parle, tout loin. J'entends le pain, papa. Tu l'entends, Sarah ? Un &lt;emphasis level="moderate"&gt;éclat de cour&lt;/emphasis&gt; glisse sur le sol. Il brille, papa. Tu le vois, près de la fenêtre ? Sarah touche l'éclat de cour. Le sol est lisse, un peu froid. Il est froid. Maman noue le lacet de Sarah. Ton lacet va là, près de la chaussure. Il tient, maman. La chaussure sent un peu la cour. Elle est froide, maman. Une boîte en fer attend sous la fenêtre. Des anneaux s'y cognent. Ça fait clic. Tu tiens ma manche, Sarah ? Oui, papa. Le tapis vert est roulé dans le coin. Un coin de laine dépasse, un peu rêche. Il est vert, maman. Il sent la laine. Ça pique un peu. Papa pose la bouteille sur l'étagère. L'eau va là. Elle est haute. La bouteille claque contre l'étagère. L'air de la cour entre un peu. J'ai les joues froides. On avance. Tu restes près de nous ? Oui, maman. Je veux le tapis, maintenant ! Tous les anneaux, d'un coup ! Tu ouvres la boîte ? Oui, papa. En ce moment, Sarah ouvre la boîte. Les anneaux sentent le fer. Ils sont froids. Sarah verse trop vite, trop fort. Les anneaux glissent sur le sol. Oh. L'éclat n'est plus là. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je les prends ! Les anneaux sont partout. Tu les vois, Sarah ? Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Claire est en classe. Un camarade s'appelle Hugo. La maîtresse explique un jeu de cubes. Hugo reste près du mur. Il a besoin de calme. Claire va &lt;emphasis&gt;répéter&lt;/emphasis&gt; la règle. Elle dit : on pose un cube. Puis un autre. Hugo va observer d'abord. Il regarde. Il ne joue pas encore. Observer d'abord, c'est possible. Plus tard, au tapis, même leçon, autre lieu. Claire répète encore. Hugo observe d'abord. Puis il pose un cube. Le soir, papa et maman écoutent. Claire dit : on peut répéter. On peut observer d'abord. Maman sourit. Papa dit : tu as laissé le temps. [pause]</t>
+          <t>Ça sent le pain chaud, près de la fenêtre. Le marché parle, tout loin. J'entends le pain, papa. Tu l'entends, Sarah ? Un &lt;emphasis&gt;éclat de cour&lt;/emphasis&gt; glisse sur le sol. Il brille, papa. Tu le vois, près de la fenêtre ? Sarah touche l'éclat de cour. Le sol est lisse, un peu froid. Il est froid. Maman noue le lacet de Sarah. Ton lacet va là, près de la chaussure. Il tient, maman. La chaussure sent un peu la cour. Elle est froide, maman. Une boîte en fer attend sous la fenêtre. Des anneaux s'y cognent. Ça fait clic. Tu tiens ma manche, Sarah ? Oui, papa. Le tapis vert est roulé dans le coin. Un coin de laine dépasse, un peu rêche. Il est vert, maman. Il sent la laine. Ça pique un peu. Papa pose la bouteille sur l'étagère. L'eau va là. Elle est haute. La bouteille claque contre l'étagère. L'air de la cour entre un peu. J'ai les joues froides. On avance. Tu restes près de nous ? Oui, maman. Je veux le tapis, maintenant ! Tous les anneaux, d'un coup ! Tu ouvres la boîte ? Oui, papa. En ce moment, Sarah ouvre la boîte. Les anneaux sentent le fer. Ils sont froids. Sarah verse trop vite, trop fort. Les anneaux glissent sur le sol. Oh. L'éclat n'est plus là. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je les prends ! Les anneaux sont partout. Tu les vois, Sarah ? Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>éclat de cour</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,52 +1326,71 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_tapis_et_les_anneaux_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La mousse du robinet sent le bois mouillé.
-narrateur|Une goutte tombe dans la bassine.
-narrateur|Elle fait un petit rond.
-narrateur|Le soleil est bas, tout orange.
-narrateur|Le cabanon a une porte peinte en vert.
-narrateur|La peinture s'écaille un peu.
-narrateur|Un bateau de bois flotte, tout léger.
-narrateur|Sa voile est un carré de tissu.
-maman|Tu as vu le rond, Sarah ?
+          <t>narrateur|Ça sent le pain chaud, près de la fenêtre.
+narrateur|Le marché parle, tout loin.
+enfant-f|J'entends le pain, papa.
+papa|Tu l'entends, Sarah ?
+narrateur|Un éclat de cour glisse sur le sol.
+enfant-f|Il brille, papa.
+papa|Tu le vois, près de la fenêtre ?
+narrateur|Sarah touche l'éclat de cour.
+narrateur|Le sol est lisse, un peu froid.
+enfant-f|Il est froid.
+narrateur|Maman noue le lacet de Sarah.
+maman|Ton lacet va là, près de la chaussure.
+enfant-f|Il tient, maman.
+narrateur|La chaussure sent un peu la cour.
+enfant-f|Elle est froide, maman.
+narrateur|Une boîte en fer attend sous la fenêtre.
+narrateur|Des anneaux s'y cognent.
+enfant-f|Ça fait clic.
+papa|Tu tiens ma manche, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Le tapis vert est roulé dans le coin.
+narrateur|Un coin de laine dépasse, un peu rêche.
+enfant-f|Il est vert, maman.
+maman|Il sent la laine.
+enfant-f|Ça pique un peu.
+narrateur|Papa pose la bouteille sur l'étagère.
+papa|L'eau va là.
+enfant-f|Elle est haute.
+narrateur|La bouteille claque contre l'étagère.
+narrateur|L'air de la cour entre un peu.
+enfant-f|J'ai les joues froides.
+papa|On avance.
+maman|Tu restes près de nous ?
 enfant-f|Oui, maman.
-enfant-f|Il grandit, puis il part.
-papa|L'eau est tiède, ce soir.
-enfant-f|Je veux qu'il traverse.
-enfant-f|Jusqu'à l'autre bord.
-maman|Avec la voile ?
-enfant-f|Oui.
-narrateur|En ce moment, Sarah touche le bateau.
-narrateur|Le bois est lisse et humide.
-narrateur|Victorino reste près de la porte.
-narrateur|Il tient le bord du cabanon.
-narrateur|Il a besoin de calme.
-enfant-f|Victorino.
-enfant-f|Tu pousses avec moi ?
-narrateur|Victorino ne vient pas encore.
-papa|On peut répéter, tout doux.
-maman|On peut observer d'abord.
-enfant-f|D'accord.
-narrateur|Une feuille tombe dans l'eau.
-narrateur|Elle devient une petite île.
-papa|Tu as vu la feuille, Sarah ?
-enfant-f|Oui.
-enfant-f|Le bateau peut tourner autour.
-maman|Oui.
-maman|Sans presser.
-narrateur|Sarah pose un doigt sur l'eau.
-narrateur|L'eau est tiède, comme papa a dit.
-narrateur|Victorino regarde depuis la porte.
-narrateur|Ses pieds restent sur la pierre.</t>
+enfant-f|Je veux le tapis, maintenant !
+enfant-f|Tous les anneaux, d'un coup !
+papa|Tu ouvres la boîte ?
+enfant-f|Oui, papa.
+narrateur|En ce moment, Sarah ouvre la boîte.
+narrateur|Les anneaux sentent le fer.
+enfant-f|Ils sont froids.
+narrateur|Sarah verse trop vite, trop fort.
+narrateur|Les anneaux glissent sur le sol.
+enfant-f|Oh.
+narrateur|L'éclat n'est plus là.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Je les prends !
+maman|Les anneaux sont partout.
+papa|Tu les vois, Sarah ?
+narrateur|Les épaules de Sarah tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>eau,bois</t>
+          <t>pain,fer</t>
         </is>
       </c>
     </row>
@@ -1398,17 +1417,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Victorino a besoin de calme. Que peut-on faire ?</t>
+          <t>Sarah a besoin de calme. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino a besoin de calme. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah a besoin de &lt;emphasis level="moderate"&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Hugo a besoin de calme. Que peut-on faire ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah a besoin de &lt;emphasis&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1433,7 +1452,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On répète la règle. Victorino peut quoi d'abord ?</t>
+          <t>On peut répéter. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1471,7 +1490,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1479,10 +1498,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1497,34 +1516,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1533,28 +1556,28 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=on_dit_le_mot_une_seconde_fois; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Victorino a besoin de calme.
+          <t>narrateur|Sarah a besoin de calme.
 narrateur|Que peut-on faire ?</t>
         </is>
       </c>
@@ -1582,17 +1605,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah va près de la porte. Elle répète, tout bas. On pousse. Puis on attend. Victorino écoute. Il va observer d'abord. Sarah pousse le bateau un peu. Elle attend. Le bateau tourne autour de la feuille. Tu as vu le tour, Victorino ? Oui. Observer d'abord, c'est possible. Victorino avance un pas. Puis il s'arrête. Il observe d'abord. La voile est mouillée, en bas. Oui. Elle tient encore. Sarah pousse encore un peu. Le bateau n'est pas à l'autre bord. Tu as répété, Sarah ? Oui, maman.</t>
+          <t>Sarah avance trop vite vers les anneaux. Tous, maintenant ! Sa voix se mélange au marché. Oh. Les anneaux restent en tas. Elle refuse de foncer. Sarah referme la main. Elle regarde le sol, un instant. Tu veux venir près de la boîte ? Papa s'accroupit à la même hauteur. Sarah pose un genou près du fer. Le fer est lisse, un peu froid. Un anneau. Puis un autre. Elle dit les mots plus bas. Un anneau. Papa dit le mot, comme elle. Puis un autre. Sarah dit le mot, une seconde fois. Merci, Sarah. Maman a entendu toute la phrase. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, papa. Sarah pose un anneau rouge. Rouge. L'anneau fait clic sur le sol. Tu le vois, celui-là ? Oui, maman. Sarah pose un anneau jaune, plus loin. Jaune. Il tient, celui-là ? Oui, papa. Un chemin d'anneaux avance vers la fenêtre. Il va vers la fenêtre. Tu le vois, le chemin ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah va près de la porte. Elle répète, tout bas. On pousse. Puis on attend. Victorino écoute. Il va observer d'abord. Sarah pousse le bateau un peu. Elle attend. Le bateau tourne autour de la feuille. Tu as vu le tour, Victorino ? Oui. Observer d'abord, c'est possible. Victorino avance un pas. Puis il s'arrête. Il observe d'abord. La voile est mouillée, en bas. Oui. Elle tient encore. Sarah pousse encore un peu. Le bateau n'est pas à l'autre bord. Tu as répété, Sarah ? Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah avance trop vite vers les anneaux. Tous, maintenant ! Sa voix se mélange au marché. Oh. Les anneaux restent en tas. Elle refuse de foncer. Sarah referme la main. Elle regarde le sol, un instant. Tu veux venir près de la boîte ? Papa s'accroupit à la même hauteur. Sarah pose un genou près du fer. Le fer est lisse, un peu froid. &lt;emphasis level="moderate"&gt;Un anneau&lt;/emphasis&gt;. Puis un autre. Elle dit les mots plus bas. Un anneau. Papa dit le mot, comme elle. Puis un autre. Sarah dit le mot, une seconde fois. Merci, Sarah. Maman a entendu toute la phrase. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, papa. Sarah pose un anneau rouge. Rouge. L'anneau fait clic sur le sol. Tu le vois, celui-là ? Oui, maman. Sarah pose un anneau jaune, plus loin. Jaune. Il tient, celui-là ? Oui, papa. Un chemin d'anneaux avance vers la fenêtre. Il va vers la fenêtre. Tu le vois, le chemin ? Oui, maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Claire a répété. Hugo a observé d'abord. Puis il a joué un peu. Papa et maman ont écouté. [pause]</t>
+          <t>Sarah avance trop vite vers les anneaux. Tous, maintenant ! Sa voix se mélange au marché. Oh. Les anneaux restent en tas. Elle refuse de foncer. Sarah referme la main. Elle regarde le sol, un instant. Tu veux venir près de la boîte ? Papa s'accroupit à la même hauteur. Sarah pose un genou près du fer. Le fer est lisse, un peu froid. &lt;emphasis&gt;Un anneau&lt;/emphasis&gt;. Puis un autre. Elle dit les mots plus bas. Un anneau. Papa dit le mot, comme elle. Puis un autre. Sarah dit le mot, une seconde fois. Merci, Sarah. Maman a entendu toute la phrase. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, papa. Sarah pose un anneau rouge. Rouge. L'anneau fait clic sur le sol. Tu le vois, celui-là ? Oui, maman. Sarah pose un anneau jaune, plus loin. Jaune. Il tient, celui-là ? Oui, papa. Un chemin d'anneaux avance vers la fenêtre. Il va vers la fenêtre. Tu le vois, le chemin ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1639,7 +1662,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1647,10 +1670,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1671,7 +1694,11 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>Un anneau</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
@@ -1683,16 +1710,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1701,10 +1728,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1717,38 +1744,54 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=la_voix_forte_echoue_le_mot_revient_plus_bas; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah va près de la porte.
-narrateur|Elle répète, tout bas.
-enfant-f|On pousse.
-enfant-f|Puis on attend.
-narrateur|Victorino écoute.
-narrateur|Il va observer d'abord.
-narrateur|Sarah pousse le bateau un peu.
-narrateur|Elle attend.
-narrateur|Le bateau tourne autour de la feuille.
-papa|Tu as vu le tour, Victorino ?
-copain|Oui.
-maman|Observer d'abord, c'est possible.
-narrateur|Victorino avance un pas.
-narrateur|Puis il s'arrête.
-narrateur|Il observe d'abord.
-enfant-f|La voile est mouillée, en bas.
-papa|Oui.
-papa|Elle tient encore.
-narrateur|Sarah pousse encore un peu.
-narrateur|Le bateau n'est pas à l'autre bord.
-maman|Tu as répété, Sarah ?
+          <t>narrateur|Sarah avance trop vite vers les anneaux.
+enfant-f|Tous, maintenant !
+narrateur|Sa voix se mélange au marché.
+enfant-f|Oh.
+narrateur|Les anneaux restent en tas.
+narrateur|Elle refuse de foncer.
+narrateur|Sarah referme la main.
+narrateur|Elle regarde le sol, un instant.
+papa|Tu veux venir près de la boîte ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Sarah pose un genou près du fer.
+narrateur|Le fer est lisse, un peu froid.
+enfant-f|Un anneau.
+enfant-f|Puis un autre.
+narrateur|Elle dit les mots plus bas.
+papa|Un anneau.
+narrateur|Papa dit le mot, comme elle.
+enfant-f|Puis un autre.
+narrateur|Sarah dit le mot, une seconde fois.
+maman|Merci, Sarah.
+narrateur|Maman a entendu toute la phrase.
+narrateur|Le ventre de Sarah se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|Tu as les mains au chaud ?
+enfant-f|Un peu, papa.
+narrateur|Sarah pose un anneau rouge.
+enfant-f|Rouge.
+narrateur|L'anneau fait clic sur le sol.
+maman|Tu le vois, celui-là ?
+enfant-f|Oui, maman.
+narrateur|Sarah pose un anneau jaune, plus loin.
+enfant-f|Jaune.
+papa|Il tient, celui-là ?
+enfant-f|Oui, papa.
+narrateur|Un chemin d'anneaux avance vers la fenêtre.
+enfant-f|Il va vers la fenêtre.
+maman|Tu le vois, le chemin ?
 enfant-f|Oui, maman.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>eau</t>
+          <t>fer,tapis</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1818,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, maman pose une serviette. La serviette est chaude de soleil. C'est un quai, tout doux. Même jeu, autre lieu. On pousse. Puis on attend. Victorino s'assoit au bord. Il observe d'abord. Puis il pose un doigt. Le bateau avance encore. Il touche l'autre bord. Il est arrivé. Moi aussi, j'ai poussé. Tu as laissé le temps, Sarah. Bravo. La voile a tenu. Une goutte reste sur le bois. On souffle ? Oui. Ils soufflent sur la voile. Le tissu tremble un peu. Tu as fini la traversée ? Oui, maman.</t>
+          <t>Sarah tire le tapis trop vite. Jusqu'à la fenêtre, d'un coup ! Le tapis se roule vers le coin. Oh. L'éclat n'est plus là. Il est parti. Sarah avance les mains. Puis elle s'arrête net. Elle refuse de foncer. Attends, je regarde. Papa attend, sans parler. Sarah observe le sol, écoute la classe. Près de la fenêtre, un éclat de cour luit. Là, près de la fenêtre. Sarah tient le tapis des deux mains. La laine est rêche, un peu froide. Elle est froide, papa. Tu le portes jusqu'à la fenêtre ? Oui, papa. On avance ? Oui, maman. Sarah déroule le tapis, sans se presser. Le tapis touche le sol froid. L'air froid revient sur les joues. Sarah serre un anneau contre elle. Il reste froid. On marche. L'anneau penche, puis se cale. Je le tiens. On avance. Sarah pose l'anneau sur la laine. Le clic est petit, près de l'éclat. Il est sur la laine. Près de la fenêtre ? Oui, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, maman pose une serviette. La serviette est chaude de soleil. C'est un quai, tout doux. Même jeu, autre lieu. On pousse. Puis on attend. Victorino s'assoit au bord. Il observe d'abord. Puis il pose un doigt. Le bateau avance encore. Il touche l'autre bord. Il est arrivé. Moi aussi, j'ai poussé. Tu as laissé le temps, Sarah. Bravo. La voile a tenu. Une goutte reste sur le bois. On souffle ? Oui. Ils soufflent sur la voile. Le tissu tremble un peu. Tu as fini la traversée ? Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah tire le tapis trop vite. Jusqu'à la fenêtre, d'un coup ! Le tapis se roule vers le coin. Oh. L'éclat n'est plus là. Il est parti. Sarah avance les mains. Puis elle s'arrête net. Elle refuse de foncer. Attends, je regarde. Papa attend, sans parler. Sarah observe le sol, écoute la classe. Près de la fenêtre, un &lt;emphasis level="moderate"&gt;éclat de cour&lt;/emphasis&gt; luit. Là, près de la fenêtre. Sarah tient le tapis des deux mains. La laine est rêche, un peu froide. Elle est froide, papa. Tu le portes jusqu'à la fenêtre ? Oui, papa. On avance ? Oui, maman. Sarah déroule le tapis, sans se presser. Le tapis touche le sol froid. L'air froid revient sur les joues. Sarah serre un anneau contre elle. Il reste froid. On marche. L'anneau penche, puis se cale. Je le tiens. On avance. Sarah pose l'anneau sur la laine. Le clic est petit, près de l'éclat. Il est sur la laine. Près de la fenêtre ? Oui, papa.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Claire range son cartable. Papa lui tend la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Sarah tire le tapis trop vite. Jusqu'à la fenêtre, d'un coup ! Le tapis se roule vers le coin. Oh. L'éclat n'est plus là. Il est parti. Sarah avance les mains. Puis elle s'arrête net. Elle refuse de foncer. Attends, je regarde. Papa attend, sans parler. Sarah observe le sol, écoute la classe. Près de la fenêtre, un &lt;emphasis&gt;éclat de cour&lt;/emphasis&gt; luit. Là, près de la fenêtre. Sarah tient le tapis des deux mains. La laine est rêche, un peu froide. Elle est froide, papa. Tu le portes jusqu'à la fenêtre ? Oui, papa. On avance ? Oui, maman. Sarah déroule le tapis, sans se presser. Le tapis touche le sol froid. L'air froid revient sur les joues. Sarah serre un anneau contre elle. Il reste froid. On marche. L'anneau penche, puis se cale. Je le tiens. On avance. Sarah pose l'anneau sur la laine. Le clic est petit, près de l'éclat. Il est sur la laine. Près de la fenêtre ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1832,7 +1875,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1840,10 +1883,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1866,30 +1909,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de cour</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1898,10 +1941,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1912,37 +1955,53 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, maman pose une serviette.
-narrateur|La serviette est chaude de soleil.
-narrateur|C'est un quai, tout doux.
-papa|Même jeu, autre lieu.
-enfant-f|On pousse.
-enfant-f|Puis on attend.
-narrateur|Victorino s'assoit au bord.
-narrateur|Il observe d'abord.
-narrateur|Puis il pose un doigt.
-narrateur|Le bateau avance encore.
-narrateur|Il touche l'autre bord.
-enfant-f|Il est arrivé.
-copain|Moi aussi, j'ai poussé.
-maman|Tu as laissé le temps, Sarah.
-papa|Bravo.
-papa|La voile a tenu.
-narrateur|Une goutte reste sur le bois.
-enfant-f|On souffle ?
-papa|Oui.
-narrateur|Ils soufflent sur la voile.
-narrateur|Le tissu tremble un peu.
-maman|Tu as fini la traversée ?
-enfant-f|Oui, maman.</t>
+          <t>narrateur|Sarah tire le tapis trop vite.
+enfant-f|Jusqu'à la fenêtre, d'un coup !
+narrateur|Le tapis se roule vers le coin.
+enfant-f|Oh.
+narrateur|L'éclat n'est plus là.
+enfant-f|Il est parti.
+narrateur|Sarah avance les mains.
+narrateur|Puis elle s'arrête net.
+narrateur|Elle refuse de foncer.
+enfant-f|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Sarah observe le sol, écoute la classe.
+narrateur|Près de la fenêtre, un éclat de cour luit.
+enfant-f|Là, près de la fenêtre.
+narrateur|Sarah tient le tapis des deux mains.
+narrateur|La laine est rêche, un peu froide.
+enfant-f|Elle est froide, papa.
+papa|Tu le portes jusqu'à la fenêtre ?
+enfant-f|Oui, papa.
+maman|On avance ?
+enfant-f|Oui, maman.
+narrateur|Sarah déroule le tapis, sans se presser.
+narrateur|Le tapis touche le sol froid.
+narrateur|L'air froid revient sur les joues.
+narrateur|Sarah serre un anneau contre elle.
+enfant-f|Il reste froid.
+papa|On marche.
+narrateur|L'anneau penche, puis se cale.
+enfant-f|Je le tiens.
+maman|On avance.
+narrateur|Sarah pose l'anneau sur la laine.
+narrateur|Le clic est petit, près de l'éclat.
+enfant-f|Il est sur la laine.
+papa|Près de la fenêtre ?
+enfant-f|Oui, papa.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>eau,tissu</t>
+          <t>tapis,fer</t>
         </is>
       </c>
     </row>
@@ -1969,17 +2028,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau repose contre le bord. On a répété. Victorino a observé d'abord. Puis il a touché l'eau. Oui. La feuille flotte encore, toute seule.</t>
+          <t>L'éclat brillait, papa. Tu le vois, comme près de la fenêtre ? Oui, un peu pâle. Sarah pose l'anneau contre le tapis. On le garde près de nous ? Oui, maman. La classe sentait le pain. Le marché est derrière nous. Un bruit de fer n'est plus aussi net. Sarah respire, plus large. On rentre ? Oui. Les joues de Sarah se réchauffent. L'anneau reste froid sous la main. Un éclat de cour reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau repose contre le bord. On a répété. Victorino a observé d'abord. Puis il a touché l'eau. Oui. La feuille flotte encore, toute seule.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'éclat brillait, papa. Tu le vois, comme près de la fenêtre ? Oui, un peu pâle. Sarah pose l'anneau contre le tapis. On le garde près de nous ? Oui, maman. La classe sentait le pain. Le marché est derrière nous. Un bruit de fer n'est plus aussi net. Sarah respire, plus large. On rentre ? Oui. Les joues de Sarah se réchauffent. L'anneau reste froid sous la main. Un &lt;emphasis level="moderate"&gt;éclat de cour&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'éclat brillait, papa. Tu le vois, comme près de la fenêtre ? Oui, un peu pâle. Sarah pose l'anneau contre le tapis. On le garde près de nous ? Oui, maman. La classe sentait le pain. Le marché est derrière nous. Un bruit de fer n'est plus aussi net. Sarah respire, plus large. On rentre ? Oui. Les joues de Sarah se réchauffent. L'anneau reste froid sous la main. Un &lt;emphasis&gt;éclat de cour&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2026,18 +2085,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2046,12 +2105,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2060,17 +2119,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cour</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2079,11 +2142,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2092,29 +2155,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le bateau repose contre le bord.
-enfant-f|On a répété.
-enfant-f|Victorino a observé d'abord.
-maman|Puis il a touché l'eau.
-papa|Oui.
-narrateur|La feuille flotte encore, toute seule.</t>
+          <t>enfant-f|L'éclat brillait, papa.
+papa|Tu le vois, comme près de la fenêtre ?
+enfant-f|Oui, un peu pâle.
+narrateur|Sarah pose l'anneau contre le tapis.
+maman|On le garde près de nous ?
+enfant-f|Oui, maman.
+enfant-f|La classe sentait le pain.
+maman|Le marché est derrière nous.
+narrateur|Un bruit de fer n'est plus aussi net.
+narrateur|Sarah respire, plus large.
+papa|On rentre ?
+enfant-f|Oui.
+narrateur|Les joues de Sarah se réchauffent.
+narrateur|L'anneau reste froid sous la main.
+narrateur|Un éclat de cour reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pain</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2213,6 +2294,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>